<commit_message>
update 762 muzzles (308 suppressor buff, adjust pbs to match, update weights)
</commit_message>
<xml_diff>
--- a/changes/308-barrels-muzzles.xlsx
+++ b/changes/308-barrels-muzzles.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C7BCEDC-4D27-44BC-80AA-81FA673A7D94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0991D43-547F-495F-A5CA-D4FCF7C4B5CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="137">
   <si>
     <t>old</t>
   </si>
@@ -149,36 +149,6 @@
     <t>HK PSG-1 Bull 650mm 7.62x51</t>
   </si>
   <si>
-    <t>fr_ordnance_mc51_211mm_7.62x51_barrel</t>
-  </si>
-  <si>
-    <t>FR Ordnance MC51 211mm 7.62x51</t>
-  </si>
-  <si>
-    <t>fr_ordnance_mc51k_145mm_7.62x51_barrel</t>
-  </si>
-  <si>
-    <t>FR Ordnance MC51k 145mm 7.62x51</t>
-  </si>
-  <si>
-    <t>fr_ordnance_mc51sd_125mm_7.62x51_barrel</t>
-  </si>
-  <si>
-    <t>FR Ordinance MC51SD 125mm 7.62x51</t>
-  </si>
-  <si>
-    <t>fr_ordnance_mc51sd_suppressor</t>
-  </si>
-  <si>
-    <t>FR Ordinance MC51SD Suppressor</t>
-  </si>
-  <si>
-    <t>hughes_precision_m15x1rh_to_5_8x24_thread_adapter</t>
-  </si>
-  <si>
-    <t>Hughes Precision M15x1RH to 5/8x24 Thread</t>
-  </si>
-  <si>
     <t>hk_bird_cage_flash_hider_m15x1rh</t>
   </si>
   <si>
@@ -191,94 +161,10 @@
     <t>DS Arms SA-58</t>
   </si>
   <si>
-    <t>dsa_sa58_305mm_barrel</t>
-  </si>
-  <si>
-    <t>DSA SA-58 12"</t>
-  </si>
-  <si>
-    <t>dsa_sa58_330mm_barrel</t>
-  </si>
-  <si>
-    <t>DSA SA-58 13"</t>
-  </si>
-  <si>
-    <t>dsa_sa58_406mm_fluted_barrel</t>
-  </si>
-  <si>
-    <t>DSA SA-58 16" Fluted</t>
-  </si>
-  <si>
-    <t>dsa_sa58_406mm_barrel</t>
-  </si>
-  <si>
-    <t>DSA SA-58 16"</t>
-  </si>
-  <si>
-    <t>dsa_sa58_457mm_barrel</t>
-  </si>
-  <si>
-    <t>DSA SA-58 18"</t>
-  </si>
-  <si>
-    <t>dsa_sa58_533mm_barrel</t>
-  </si>
-  <si>
-    <t>DSA SA-58 21"</t>
-  </si>
-  <si>
     <t>SCARH</t>
   </si>
   <si>
     <t>FN SCAR Mk17</t>
-  </si>
-  <si>
-    <t>hi_desertdog_hdd_tactical_scarh_267mm_7.62x51_barrel</t>
-  </si>
-  <si>
-    <t>Hi-desertdog HDD Tactical Scar H 267mm Barrel</t>
-  </si>
-  <si>
-    <t>fn_scar_h_330mm_barrel</t>
-  </si>
-  <si>
-    <t>FN SCAR-H 330mm</t>
-  </si>
-  <si>
-    <t>fn_scar_h_406mm_barrel</t>
-  </si>
-  <si>
-    <t>FN SCAR-H 406mm</t>
-  </si>
-  <si>
-    <t>deadshot_scar20_spiral_406mm_threaded_barrel</t>
-  </si>
-  <si>
-    <t>Deadshot FN SCAR 20 Spiral 16" Threaded</t>
-  </si>
-  <si>
-    <t>fn_scar_h_508mm_barrel</t>
-  </si>
-  <si>
-    <t>FN SCAR-H 508mm</t>
-  </si>
-  <si>
-    <t>deadshot_scar20_spiral_508mm_threaded_barrel</t>
-  </si>
-  <si>
-    <t>Deadshot FN SCAR 20 Spiral 20" Threaded</t>
-  </si>
-  <si>
-    <t>fn_scar_mk20_508mm_barrel</t>
-  </si>
-  <si>
-    <t>FN SCAR Mk20 508mm</t>
-  </si>
-  <si>
-    <t>dsa_3prong_trident_7.62x51_flash_hider</t>
-  </si>
-  <si>
-    <t>DSA 3-Prong Trident 7.62x51</t>
   </si>
   <si>
     <t>fn_fal_austrian_7.62x51_stg58_flash_hider</t>
@@ -293,40 +179,16 @@
     <t>FN FAL Belgian Style 7.62x51</t>
   </si>
   <si>
-    <t>rhodesian_halbek_muzzle_device</t>
-  </si>
-  <si>
-    <t>Rhodesian Reproduction Halbek</t>
-  </si>
-  <si>
-    <t>fn_scar17_7.62x51_3prong_european_flash_hider</t>
-  </si>
-  <si>
-    <t>FN Scar Mk17 .308 3-Prong European</t>
-  </si>
-  <si>
-    <t>aac_scar_sd_blackout_51_tooth_flashhider_supp_mount</t>
-  </si>
-  <si>
-    <t>AAC SCAR-SD Blackout 51-Tooth Flash Hider</t>
-  </si>
-  <si>
     <t>lantac_dgn762b_asr_muzzle_brake</t>
   </si>
   <si>
     <t>LANTAC DGM762B-ASR Muzzle Brake</t>
   </si>
   <si>
-    <t>surefire_socom762_sfmb_muzzle_brake</t>
+    <t>rhodesian_halbek_muzzle_device</t>
   </si>
   <si>
-    <t>Surefire SOCOM762 SFMB Muzzle Break</t>
-  </si>
-  <si>
-    <t>strike_industries_jcomp_gen2_7.62x51_muzzle_brake</t>
-  </si>
-  <si>
-    <t>Strike Industries JCOMP Gen2 7.62x51 Muzzle Brake</t>
+    <t>Rhodesian Reproduction Halbek</t>
   </si>
   <si>
     <t>tiger_rock_ar10_7.62x51_barrett_style_muzzle_brake_with_jam_nut</t>
@@ -335,46 +197,10 @@
     <t>Tiger Rock AR-10 .308 Barrett Style Muzzle Brake with Jam Nut</t>
   </si>
   <si>
-    <t>surefire_warden_blast_regulator</t>
-  </si>
-  <si>
-    <t>Surefire Warden Blast Regulator</t>
-  </si>
-  <si>
-    <t>strike_industries_oppressor_blast_shield</t>
-  </si>
-  <si>
-    <t>Strike Industries Oppressor Blast Shield</t>
-  </si>
-  <si>
     <t>sig_srd762ti_suppressor</t>
   </si>
   <si>
     <t>Sig SRD762Ti</t>
-  </si>
-  <si>
-    <t>oss_bpr_suppressor_system_bpr_1425</t>
-  </si>
-  <si>
-    <t>OSS BPR Suppressor System BPR-1425</t>
-  </si>
-  <si>
-    <t>oss_bpr_suppressor_system_srm_6</t>
-  </si>
-  <si>
-    <t>OSS BPR Suppressor System SRM-6</t>
-  </si>
-  <si>
-    <t>silencerco_osprey45_gen1_45acp_suppressor_7.62x51_piston</t>
-  </si>
-  <si>
-    <t>SilencerCo Osprey 45 Gen 1 .45ACP Suppressor w/ 7.62x51 Piston</t>
-  </si>
-  <si>
-    <t>silencerco_osprey45_gen1_45acp_suppressor_7.62x51_piston_flipped</t>
-  </si>
-  <si>
-    <t>SilencerCo Osprey 45 Gen 1 .45ACP Suppressor w/ 7.62x51 Piston Flipped</t>
   </si>
   <si>
     <t>odin_works_tiduro_.338_modular_no_baffle_suppressor</t>
@@ -407,18 +233,6 @@
     <t>Odin Works Tiduro Thread Adaptor Module</t>
   </si>
   <si>
-    <t>silencerco_omega_300_suppressor</t>
-  </si>
-  <si>
-    <t>SilencerCo OMEGA 300</t>
-  </si>
-  <si>
-    <t>silencerco_qd_asr_mount</t>
-  </si>
-  <si>
-    <t>SilencerCo QD ASR Mount</t>
-  </si>
-  <si>
     <t>ips_7.62x51_1inch_barrel_extension</t>
   </si>
   <si>
@@ -437,19 +251,199 @@
     <t>IPS 7.62x51 4in Barrel Extension</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
+    <t>ferro_ordnance_mc51_211mm_7.62x51_barrel</t>
   </si>
   <si>
-    <t>dsa_warz_series_7.62x51_flash_hider</t>
+    <t>FR Ordnance MC51 211mm 7.62x51</t>
   </si>
   <si>
-    <t>DSA WarZ Series 7.62x51</t>
+    <t>ferro_ordnance_mc51k_145mm_7.62x51_barrel</t>
   </si>
   <si>
-    <t>dsa_sa58_210mm_premium_pistol_barrel</t>
+    <t>FR Ordnance MC51k 145mm 7.62x51</t>
   </si>
   <si>
-    <t>DSA SA-58 8.25" Premium Pistol</t>
+    <t>ferro_ordnance_mc51sd_125mm_7.62x51_barrel</t>
+  </si>
+  <si>
+    <t>FR Ordinance MC51SD 125mm 7.62x51</t>
+  </si>
+  <si>
+    <t>ferro_ordnance_mc51sd_suppressor</t>
+  </si>
+  <si>
+    <t>FR Ordinance MC51SD Suppressor</t>
+  </si>
+  <si>
+    <t>tubewerx_m15x1rh_to_5_8x24_thread_adapter</t>
+  </si>
+  <si>
+    <t>Hughes Precision M15x1RH to 5/8x24 Thread</t>
+  </si>
+  <si>
+    <t>rsa_sa58_210mm_premium_pistol_barrel</t>
+  </si>
+  <si>
+    <t>RSA SA-58 8.25"" Premium Pistol</t>
+  </si>
+  <si>
+    <t>rsa_sa58_305mm_barrel</t>
+  </si>
+  <si>
+    <t>RSA SA-58 12"</t>
+  </si>
+  <si>
+    <t>rsa_sa58_330mm_barrel</t>
+  </si>
+  <si>
+    <t>RSA SA-58 13"</t>
+  </si>
+  <si>
+    <t>rsa_sa58_406mm_fluted_barrel</t>
+  </si>
+  <si>
+    <t>DSA SA-58 16" Fluted</t>
+  </si>
+  <si>
+    <t>rsa_sa58_406mm_barrel</t>
+  </si>
+  <si>
+    <t>DSA SA-58 16"</t>
+  </si>
+  <si>
+    <t>rsa_sa58_457mm_barrel</t>
+  </si>
+  <si>
+    <t>DSA SA-58 18"</t>
+  </si>
+  <si>
+    <t>rsa_sa58_533mm_barrel</t>
+  </si>
+  <si>
+    <t>DSA SA-58 21"</t>
+  </si>
+  <si>
+    <t>hi_dog_hdd_tactical_scarh_267mm_7.62x51_barrel</t>
+  </si>
+  <si>
+    <t>Hi-desertdog HDD Tactical Scar H 267mm Barrel</t>
+  </si>
+  <si>
+    <t>aft_mk_17_330mm_barrel</t>
+  </si>
+  <si>
+    <t>AFT Mk20 330mm</t>
+  </si>
+  <si>
+    <t>aft_mk_17_406mm_barrel</t>
+  </si>
+  <si>
+    <t>AFT Mk20 406mm</t>
+  </si>
+  <si>
+    <t>barreltech_scar20_spiral_406mm_threaded_barrel</t>
+  </si>
+  <si>
+    <t>Deadshot FN SCAR 20 Spiral 16" Threaded</t>
+  </si>
+  <si>
+    <t>aft_mk_17_508mm_barrel</t>
+  </si>
+  <si>
+    <t>AFT Mk20 508mm</t>
+  </si>
+  <si>
+    <t>barreltech_scar20_spiral_508mm_threaded_barrel</t>
+  </si>
+  <si>
+    <t>Deadshot FN SCAR 20 Spiral 20" Threaded</t>
+  </si>
+  <si>
+    <t>aft_mk20_508mm_barrel</t>
+  </si>
+  <si>
+    <t>rsa_3prong_trident_7.62x51_flash_hider</t>
+  </si>
+  <si>
+    <t>RSA 3-Prong Trident 7.62x51</t>
+  </si>
+  <si>
+    <t>rsa_warz_series_7.62x51_flash_hider</t>
+  </si>
+  <si>
+    <t>RSA WarZ Series 7.62x51</t>
+  </si>
+  <si>
+    <t>aft17_7.62x51_3prong_european_flash_hider</t>
+  </si>
+  <si>
+    <t>FN Scar Mk17 .308 3-Prong European</t>
+  </si>
+  <si>
+    <t>ewc_scar_sd_blackout_51_tooth_flashhider_supp_mount</t>
+  </si>
+  <si>
+    <t>AAC SCAR-SD Blackout 51-Tooth Flash Hider</t>
+  </si>
+  <si>
+    <t>centrefire_socom762_sfmb_muzzle_brake</t>
+  </si>
+  <si>
+    <t>Surefire SOCOM762 SFMB Muzzle Break</t>
+  </si>
+  <si>
+    <t>smite_industries_jcomp_gen2_7.62x51_muzzle_brake</t>
+  </si>
+  <si>
+    <t>Strike Industries JCOMP Gen2 7.62x51 Muzzle Brake</t>
+  </si>
+  <si>
+    <t>centrefire_warden_blast_regulator</t>
+  </si>
+  <si>
+    <t>Centrefire Warden Blast Regulator</t>
+  </si>
+  <si>
+    <t>smite_industries_oppressor_blast_shield</t>
+  </si>
+  <si>
+    <t>Strike Industries Oppressor Blast Shield</t>
+  </si>
+  <si>
+    <t>spiderweb_bpr_suppressor_system_bpr_1425</t>
+  </si>
+  <si>
+    <t>OSS BPR Suppressor System BPR-1425</t>
+  </si>
+  <si>
+    <t>spiderweb_bpr_suppressor_system_srm_6</t>
+  </si>
+  <si>
+    <t>OSS BPR Suppressor System SRM-6</t>
+  </si>
+  <si>
+    <t>suppressors_inc_osprey45_gen1_45acp_suppressor_7.62x51_piston</t>
+  </si>
+  <si>
+    <t>SilencerCo Osprey 45 Gen 1 .45ACP Suppressor w/ 7.62x51 Piston</t>
+  </si>
+  <si>
+    <t>suppressors_inc_osprey45_gen1_45acp_suppressor_7.62x51_piston_flipped</t>
+  </si>
+  <si>
+    <t>SilencerCo Osprey 45 Gen 1 .45ACP Suppressor w/ 7.62x51 Piston Flipped</t>
+  </si>
+  <si>
+    <t>suppressors_inc_omega_300_suppressor</t>
+  </si>
+  <si>
+    <t>SilencerCo OMEGA 300</t>
+  </si>
+  <si>
+    <t>suppressors_inc_qd_asr_mount</t>
+  </si>
+  <si>
+    <t>SilencerCo QD ASR Mount</t>
   </si>
 </sst>
 </file>
@@ -461,7 +455,6 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -509,8 +502,7 @@
   <dxfs count="1">
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC9DAF8"/>
+        <patternFill>
           <bgColor rgb="FFC9DAF8"/>
         </patternFill>
       </fill>
@@ -569,11 +561,11 @@
         <a:srgbClr val="0563C1"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Sheets">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -581,7 +573,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Sheets">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -590,23 +582,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
                 <a:lumMod val="110000"/>
                 <a:satMod val="105000"/>
-                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="103000"/>
-                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="109000"/>
-                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -616,23 +608,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
                 <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
                 <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
                 <a:lumMod val="99000"/>
                 <a:satMod val="120000"/>
-                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -640,26 +632,23 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -694,17 +683,17 @@
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
+                <a:satMod val="150000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
@@ -727,7 +716,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AI1027"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
     <col min="2" max="2" width="65.140625" customWidth="1"/>
@@ -923,15 +912,14 @@
         <v>65000</v>
       </c>
       <c r="N3" s="2">
-        <f t="shared" ref="N3:N68" si="1">C3-D3*20-E3*0.8-F3*0.6-H3*15+I3*40+J3/300</f>
-        <v>-138.06666666666666</v>
+        <v>-138.07</v>
       </c>
       <c r="O3" s="1"/>
       <c r="P3" s="1">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="Q3" s="1">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="R3" s="1">
         <v>80</v>
@@ -943,7 +931,7 @@
         <v>0</v>
       </c>
       <c r="U3" s="1">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
       <c r="V3" s="1">
         <v>1</v>
@@ -957,8 +945,8 @@
         <v>65000</v>
       </c>
       <c r="AA3" s="2">
-        <f t="shared" ref="AA3:AA68" si="2">P3-Q3*20-R3*0.8-S3*0.6-U3*15+V3*40+W3/300</f>
-        <v>-75.666666666666671</v>
+        <f t="shared" ref="AA3:AA68" si="1">P3-Q3*20-R3*0.8-S3*0.6-U3*15+V3*40+W3/300</f>
+        <v>-71.416666666666671</v>
       </c>
       <c r="AB3" s="1"/>
       <c r="AC3" s="1"/>
@@ -1000,15 +988,14 @@
         <v>500</v>
       </c>
       <c r="N4" s="2">
-        <f t="shared" si="1"/>
-        <v>-6.1833333333333327</v>
+        <v>-6.18</v>
       </c>
       <c r="O4" s="1"/>
       <c r="P4" s="1">
         <v>0</v>
       </c>
       <c r="Q4" s="1">
-        <v>1.02</v>
+        <v>1.32</v>
       </c>
       <c r="R4" s="1">
         <v>0</v>
@@ -1018,7 +1005,7 @@
       </c>
       <c r="T4" s="1"/>
       <c r="U4" s="1">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="V4" s="1">
         <v>0</v>
@@ -1029,11 +1016,11 @@
       <c r="X4" s="1"/>
       <c r="Y4" s="1"/>
       <c r="Z4" s="1">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="AA4" s="2">
-        <f t="shared" si="2"/>
-        <v>-24.15</v>
+        <f t="shared" si="1"/>
+        <v>-26.400000000000002</v>
       </c>
       <c r="AB4" s="1"/>
       <c r="AC4" s="1"/>
@@ -1047,7 +1034,7 @@
       </c>
       <c r="AH4" s="1"/>
       <c r="AI4" s="1">
-        <f t="shared" ref="AI4:AI36" si="3">AF4+AG4*0.038+AH4</f>
+        <f t="shared" ref="AI4:AI36" si="2">AF4+AG4*0.038+AH4</f>
         <v>0.92086679999999999</v>
       </c>
     </row>
@@ -1086,31 +1073,30 @@
         <v>1000</v>
       </c>
       <c r="N5" s="2">
-        <f t="shared" si="1"/>
-        <v>-10.966666666666667</v>
+        <v>-10.97</v>
       </c>
       <c r="O5" s="1"/>
       <c r="P5" s="1">
         <v>-1</v>
       </c>
       <c r="Q5" s="1">
-        <v>1.02</v>
+        <v>1.32</v>
       </c>
       <c r="R5" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S5" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T5" s="1"/>
       <c r="U5" s="1">
-        <v>0.35</v>
+        <v>0.1</v>
       </c>
       <c r="V5" s="1">
         <v>0</v>
       </c>
       <c r="W5" s="1">
-        <v>-50</v>
+        <v>0</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="1"/>
@@ -1118,8 +1104,8 @@
         <v>1000</v>
       </c>
       <c r="AA5" s="2">
-        <f t="shared" si="2"/>
-        <v>-29.616666666666667</v>
+        <f t="shared" si="1"/>
+        <v>-30.300000000000004</v>
       </c>
       <c r="AB5" s="1"/>
       <c r="AC5" s="1"/>
@@ -1133,7 +1119,7 @@
       </c>
       <c r="AH5" s="1"/>
       <c r="AI5" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.92086679999999999</v>
       </c>
     </row>
@@ -1172,8 +1158,7 @@
         <v>0</v>
       </c>
       <c r="N6" s="2">
-        <f t="shared" si="1"/>
-        <v>9.1166666666666654</v>
+        <v>9.1199999999999992</v>
       </c>
       <c r="O6" s="3"/>
       <c r="P6" s="1">
@@ -1204,7 +1189,7 @@
         <v>0</v>
       </c>
       <c r="AA6" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>14.416666666666666</v>
       </c>
       <c r="AB6" s="1"/>
@@ -1215,7 +1200,7 @@
       <c r="AG6" s="1"/>
       <c r="AH6" s="1"/>
       <c r="AI6" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -1234,7 +1219,6 @@
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
       <c r="N7" s="2">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O7" s="1"/>
@@ -1250,7 +1234,7 @@
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
       <c r="AA7" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AB7" s="1"/>
@@ -1261,7 +1245,7 @@
       <c r="AG7" s="1"/>
       <c r="AH7" s="1"/>
       <c r="AI7" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -1302,8 +1286,7 @@
         <v>30000</v>
       </c>
       <c r="N8" s="2">
-        <f t="shared" si="1"/>
-        <v>-52.483333333333341</v>
+        <v>-52.48</v>
       </c>
       <c r="O8" s="1"/>
       <c r="P8" s="4">
@@ -1313,7 +1296,7 @@
         <v>0</v>
       </c>
       <c r="R8" s="4">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="S8" s="4">
         <v>100</v>
@@ -1336,8 +1319,8 @@
         <v>30000</v>
       </c>
       <c r="AA8" s="2">
-        <f t="shared" si="2"/>
-        <v>-43.583333333333336</v>
+        <f t="shared" si="1"/>
+        <v>-35.583333333333336</v>
       </c>
       <c r="AB8" s="1"/>
       <c r="AC8" s="1"/>
@@ -1347,7 +1330,7 @@
       <c r="AG8" s="1"/>
       <c r="AH8" s="1"/>
       <c r="AI8" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -1386,8 +1369,7 @@
         <v>0</v>
       </c>
       <c r="N9" s="2">
-        <f t="shared" si="1"/>
-        <v>-11.766666666666667</v>
+        <v>-11.77</v>
       </c>
       <c r="O9" s="1"/>
       <c r="P9" s="4">
@@ -1418,7 +1400,7 @@
         <v>0</v>
       </c>
       <c r="AA9" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-15.96666666666667</v>
       </c>
       <c r="AB9" s="1"/>
@@ -1433,7 +1415,7 @@
       </c>
       <c r="AH9" s="1"/>
       <c r="AI9" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.7074033999999999</v>
       </c>
     </row>
@@ -1472,8 +1454,7 @@
         <v>800</v>
       </c>
       <c r="N10" s="2">
-        <f t="shared" si="1"/>
-        <v>-5.1233333333333313</v>
+        <v>-5.12</v>
       </c>
       <c r="O10" s="1"/>
       <c r="P10" s="4">
@@ -1504,7 +1485,7 @@
         <v>800</v>
       </c>
       <c r="AA10" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-16.023333333333333</v>
       </c>
       <c r="AB10" s="1"/>
@@ -1519,7 +1500,7 @@
       </c>
       <c r="AH10" s="1"/>
       <c r="AI10" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.78369979999999995</v>
       </c>
     </row>
@@ -1558,8 +1539,7 @@
         <v>4800</v>
       </c>
       <c r="N11" s="2">
-        <f t="shared" si="1"/>
-        <v>-5.3333333333333321</v>
+        <v>-5.33</v>
       </c>
       <c r="O11" s="1"/>
       <c r="P11" s="4">
@@ -1590,7 +1570,7 @@
         <v>4800</v>
       </c>
       <c r="AA11" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-15.68333333333333</v>
       </c>
       <c r="AB11" s="1"/>
@@ -1605,7 +1585,7 @@
       </c>
       <c r="AH11" s="1"/>
       <c r="AI11" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.99763599999999997</v>
       </c>
     </row>
@@ -1644,8 +1624,7 @@
         <v>4500</v>
       </c>
       <c r="N12" s="2">
-        <f t="shared" si="1"/>
-        <v>1.2966666666666682</v>
+        <v>1.3</v>
       </c>
       <c r="O12" s="1"/>
       <c r="P12" s="4">
@@ -1676,7 +1655,7 @@
         <v>4500</v>
       </c>
       <c r="AA12" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-14.453333333333328</v>
       </c>
       <c r="AB12" s="1"/>
@@ -1691,16 +1670,16 @@
       </c>
       <c r="AH12" s="1"/>
       <c r="AI12" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1.0724427999999999</v>
       </c>
     </row>
     <row r="13" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>38</v>
+        <v>72</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="C13" s="4">
         <v>8</v>
@@ -1730,8 +1709,7 @@
         <v>3500</v>
       </c>
       <c r="N13" s="2">
-        <f t="shared" si="1"/>
-        <v>-17.203333333333333</v>
+        <v>-17.2</v>
       </c>
       <c r="O13" s="1"/>
       <c r="P13" s="4">
@@ -1762,7 +1740,7 @@
         <v>3500</v>
       </c>
       <c r="AA13" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-28.45333333333333</v>
       </c>
       <c r="AB13" s="1"/>
@@ -1777,16 +1755,16 @@
       </c>
       <c r="AH13" s="1"/>
       <c r="AI13" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.41566942000000007</v>
       </c>
     </row>
     <row r="14" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>40</v>
+        <v>74</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>41</v>
+        <v>75</v>
       </c>
       <c r="C14" s="4">
         <v>14</v>
@@ -1816,8 +1794,7 @@
         <v>1500</v>
       </c>
       <c r="N14" s="2">
-        <f t="shared" si="1"/>
-        <v>-20.870000000000005</v>
+        <v>-20.87</v>
       </c>
       <c r="O14" s="1"/>
       <c r="P14" s="4">
@@ -1848,7 +1825,7 @@
         <v>1500</v>
       </c>
       <c r="AA14" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-18.52</v>
       </c>
       <c r="AB14" s="1"/>
@@ -1863,16 +1840,16 @@
       </c>
       <c r="AH14" s="1"/>
       <c r="AI14" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.31692907999999997</v>
       </c>
     </row>
     <row r="15" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="C15" s="4">
         <v>16</v>
@@ -1902,8 +1879,7 @@
         <v>2500</v>
       </c>
       <c r="N15" s="2">
-        <f t="shared" si="1"/>
-        <v>-18.473333333333333</v>
+        <v>-18.47</v>
       </c>
       <c r="O15" s="1"/>
       <c r="P15" s="4">
@@ -1934,7 +1910,7 @@
         <v>2500</v>
       </c>
       <c r="AA15" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-29.573333333333331</v>
       </c>
       <c r="AB15" s="1"/>
@@ -1949,16 +1925,16 @@
       </c>
       <c r="AH15" s="1"/>
       <c r="AI15" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.28700787999999999</v>
       </c>
     </row>
     <row r="16" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>44</v>
+        <v>78</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>45</v>
+        <v>79</v>
       </c>
       <c r="C16" s="4">
         <v>-7</v>
@@ -1988,7 +1964,6 @@
         <v>5000</v>
       </c>
       <c r="N16" s="2">
-        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="O16" s="1"/>
@@ -2020,7 +1995,7 @@
         <v>5000</v>
       </c>
       <c r="AA16" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>5.0000000000000009</v>
       </c>
       <c r="AB16" s="1"/>
@@ -2031,16 +2006,16 @@
       <c r="AG16" s="1"/>
       <c r="AH16" s="1"/>
       <c r="AI16" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>46</v>
+        <v>80</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>47</v>
+        <v>81</v>
       </c>
       <c r="C17" s="1">
         <v>-1</v>
@@ -2070,8 +2045,7 @@
         <v>1000</v>
       </c>
       <c r="N17" s="2">
-        <f t="shared" si="1"/>
-        <v>-7.4666666666666668</v>
+        <v>-7.47</v>
       </c>
       <c r="O17" s="1"/>
       <c r="P17" s="1">
@@ -2102,7 +2076,7 @@
         <v>1000</v>
       </c>
       <c r="AA17" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-5.0666666666666673</v>
       </c>
       <c r="AB17" s="1"/>
@@ -2113,16 +2087,16 @@
       <c r="AG17" s="1"/>
       <c r="AH17" s="1"/>
       <c r="AI17" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C18" s="1">
         <v>-2</v>
@@ -2152,8 +2126,7 @@
         <v>0</v>
       </c>
       <c r="N18" s="2">
-        <f t="shared" si="1"/>
-        <v>6.9666666666666677</v>
+        <v>6.97</v>
       </c>
       <c r="O18" s="1"/>
       <c r="P18" s="1">
@@ -2184,7 +2157,7 @@
         <v>0</v>
       </c>
       <c r="AA18" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>14.366666666666665</v>
       </c>
       <c r="AB18" s="1"/>
@@ -2195,7 +2168,7 @@
       <c r="AG18" s="1"/>
       <c r="AH18" s="1"/>
       <c r="AI18" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2214,7 +2187,6 @@
       <c r="L19" s="1"/>
       <c r="M19" s="1"/>
       <c r="N19" s="2">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O19" s="1"/>
@@ -2230,7 +2202,7 @@
       <c r="Y19" s="1"/>
       <c r="Z19" s="1"/>
       <c r="AA19" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AB19" s="1"/>
@@ -2241,16 +2213,16 @@
       <c r="AG19" s="1"/>
       <c r="AH19" s="1"/>
       <c r="AI19" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C20" s="4">
         <v>41</v>
@@ -2282,12 +2254,11 @@
         <v>20000</v>
       </c>
       <c r="N20" s="2">
-        <f t="shared" si="1"/>
-        <v>-67.533333333333346</v>
+        <v>-67.53</v>
       </c>
       <c r="O20" s="1"/>
       <c r="P20" s="4">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="Q20" s="4">
         <v>0.75</v>
@@ -2316,8 +2287,8 @@
         <v>20000</v>
       </c>
       <c r="AA20" s="2">
-        <f t="shared" si="2"/>
-        <v>-85.083333333333329</v>
+        <f t="shared" si="1"/>
+        <v>-95.083333333333329</v>
       </c>
       <c r="AB20" s="1"/>
       <c r="AC20" s="1"/>
@@ -2327,16 +2298,16 @@
       <c r="AG20" s="1"/>
       <c r="AH20" s="1"/>
       <c r="AI20" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>137</v>
+        <v>82</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>138</v>
+        <v>83</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
@@ -2350,15 +2321,14 @@
       <c r="L21" s="3"/>
       <c r="M21" s="4"/>
       <c r="N21" s="2">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O21" s="1"/>
       <c r="P21" s="4">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="Q21" s="4">
-        <v>0.56999999999999995</v>
+        <v>0.49</v>
       </c>
       <c r="R21" s="4">
         <v>9</v>
@@ -2371,7 +2341,7 @@
         <v>0.25</v>
       </c>
       <c r="V21" s="4">
-        <v>-0.09</v>
+        <v>-0.08</v>
       </c>
       <c r="W21" s="4">
         <v>-158</v>
@@ -2382,8 +2352,8 @@
         <v>1000</v>
       </c>
       <c r="AA21" s="2">
-        <f t="shared" si="2"/>
-        <v>-18.876666666666665</v>
+        <f t="shared" si="1"/>
+        <v>-13.876666666666669</v>
       </c>
       <c r="AB21" s="1"/>
       <c r="AC21" s="1"/>
@@ -2397,16 +2367,16 @@
       </c>
       <c r="AH21" s="1"/>
       <c r="AI21" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.47350000000000003</v>
       </c>
     </row>
     <row r="22" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="C22" s="4">
         <v>12</v>
@@ -2436,15 +2406,14 @@
         <v>750</v>
       </c>
       <c r="N22" s="2">
-        <f t="shared" si="1"/>
-        <v>-16.786666666666669</v>
+        <v>-16.79</v>
       </c>
       <c r="O22" s="1"/>
       <c r="P22" s="4">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="Q22" s="4">
-        <v>0.75</v>
+        <v>0.64</v>
       </c>
       <c r="R22" s="4">
         <v>6</v>
@@ -2468,8 +2437,8 @@
         <v>750</v>
       </c>
       <c r="AA22" s="2">
-        <f t="shared" si="2"/>
-        <v>-19.486666666666665</v>
+        <f t="shared" si="1"/>
+        <v>-15.286666666666669</v>
       </c>
       <c r="AB22" s="1"/>
       <c r="AC22" s="1"/>
@@ -2483,16 +2452,16 @@
       </c>
       <c r="AH22" s="1"/>
       <c r="AI22" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.65599999999999992</v>
       </c>
     </row>
     <row r="23" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>55</v>
+        <v>87</v>
       </c>
       <c r="C23" s="4">
         <v>6</v>
@@ -2522,15 +2491,14 @@
         <v>500</v>
       </c>
       <c r="N23" s="2">
-        <f t="shared" si="1"/>
-        <v>-15.870000000000001</v>
+        <v>-15.87</v>
       </c>
       <c r="O23" s="1"/>
       <c r="P23" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q23" s="4">
-        <v>0.79</v>
+        <v>0.72</v>
       </c>
       <c r="R23" s="4">
         <v>4</v>
@@ -2554,8 +2522,8 @@
         <v>500</v>
       </c>
       <c r="AA23" s="2">
-        <f t="shared" si="2"/>
-        <v>-18.77</v>
+        <f t="shared" si="1"/>
+        <v>-16.369999999999997</v>
       </c>
       <c r="AB23" s="1"/>
       <c r="AC23" s="1"/>
@@ -2569,16 +2537,16 @@
       </c>
       <c r="AH23" s="1"/>
       <c r="AI23" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.69399999999999995</v>
       </c>
     </row>
     <row r="24" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>57</v>
+        <v>89</v>
       </c>
       <c r="C24" s="4">
         <v>0</v>
@@ -2608,8 +2576,7 @@
         <v>400</v>
       </c>
       <c r="N24" s="2">
-        <f t="shared" si="1"/>
-        <v>-17.29666666666667</v>
+        <v>-17.3</v>
       </c>
       <c r="O24" s="1"/>
       <c r="P24" s="4">
@@ -2640,7 +2607,7 @@
         <v>400</v>
       </c>
       <c r="AA24" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-18.446666666666669</v>
       </c>
       <c r="AB24" s="1"/>
@@ -2655,16 +2622,16 @@
       </c>
       <c r="AH24" s="1"/>
       <c r="AI24" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.80800000000000005</v>
       </c>
     </row>
     <row r="25" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>58</v>
+        <v>90</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>59</v>
+        <v>91</v>
       </c>
       <c r="C25" s="4">
         <v>-6</v>
@@ -2694,8 +2661,7 @@
         <v>0</v>
       </c>
       <c r="N25" s="2">
-        <f t="shared" si="1"/>
-        <v>-19.813333333333333</v>
+        <v>-19.809999999999999</v>
       </c>
       <c r="O25" s="1"/>
       <c r="P25" s="4">
@@ -2726,7 +2692,7 @@
         <v>0</v>
       </c>
       <c r="AA25" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-18.963333333333331</v>
       </c>
       <c r="AB25" s="1"/>
@@ -2741,16 +2707,16 @@
       </c>
       <c r="AH25" s="1"/>
       <c r="AI25" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.85799999999999998</v>
       </c>
     </row>
     <row r="26" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>60</v>
+        <v>92</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>61</v>
+        <v>93</v>
       </c>
       <c r="C26" s="4">
         <v>-14</v>
@@ -2780,8 +2746,7 @@
         <v>750</v>
       </c>
       <c r="N26" s="2">
-        <f t="shared" si="1"/>
-        <v>-16.523333333333333</v>
+        <v>-16.52</v>
       </c>
       <c r="O26" s="1"/>
       <c r="P26" s="4">
@@ -2812,7 +2777,7 @@
         <v>750</v>
       </c>
       <c r="AA26" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-18.623333333333335</v>
       </c>
       <c r="AB26" s="1"/>
@@ -2827,16 +2792,16 @@
       </c>
       <c r="AH26" s="1"/>
       <c r="AI26" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.93399999999999994</v>
       </c>
     </row>
     <row r="27" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>62</v>
+        <v>94</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>63</v>
+        <v>95</v>
       </c>
       <c r="C27" s="4">
         <v>-20</v>
@@ -2866,8 +2831,7 @@
         <v>1000</v>
       </c>
       <c r="N27" s="2">
-        <f t="shared" si="1"/>
-        <v>-20.456666666666663</v>
+        <v>-20.46</v>
       </c>
       <c r="O27" s="1"/>
       <c r="P27" s="4">
@@ -2898,7 +2862,7 @@
         <v>1000</v>
       </c>
       <c r="AA27" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-18.65666666666667</v>
       </c>
       <c r="AB27" s="1"/>
@@ -2913,7 +2877,7 @@
       </c>
       <c r="AH27" s="1"/>
       <c r="AI27" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1.048</v>
       </c>
     </row>
@@ -2932,7 +2896,6 @@
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
       <c r="N28" s="2">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O28" s="3"/>
@@ -2948,7 +2911,7 @@
       <c r="Y28" s="1"/>
       <c r="Z28" s="1"/>
       <c r="AA28" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AB28" s="1"/>
@@ -2959,16 +2922,16 @@
       <c r="AG28" s="1"/>
       <c r="AH28" s="1"/>
       <c r="AI28" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="C29" s="4">
         <v>16</v>
@@ -3000,12 +2963,11 @@
         <v>75000</v>
       </c>
       <c r="N29" s="2">
-        <f t="shared" si="1"/>
         <v>-53.5</v>
       </c>
       <c r="O29" s="1"/>
       <c r="P29" s="4">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="Q29" s="4">
         <v>0</v>
@@ -3020,7 +2982,7 @@
         <v>0</v>
       </c>
       <c r="U29" s="4">
-        <v>0.55000000000000004</v>
+        <v>0.6</v>
       </c>
       <c r="V29" s="4">
         <v>1</v>
@@ -3034,8 +2996,8 @@
         <v>75000</v>
       </c>
       <c r="AA29" s="2">
-        <f t="shared" si="2"/>
-        <v>-55.75</v>
+        <f t="shared" si="1"/>
+        <v>-66.5</v>
       </c>
       <c r="AB29" s="1"/>
       <c r="AC29" s="1"/>
@@ -3045,16 +3007,16 @@
       <c r="AG29" s="1"/>
       <c r="AH29" s="1"/>
       <c r="AI29" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>66</v>
+        <v>96</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="C30" s="4">
         <v>24</v>
@@ -3086,8 +3048,7 @@
         <v>1500</v>
       </c>
       <c r="N30" s="2">
-        <f t="shared" si="1"/>
-        <v>-9.3733333333333331</v>
+        <v>-9.3699999999999992</v>
       </c>
       <c r="O30" s="1"/>
       <c r="P30" s="4">
@@ -3107,7 +3068,7 @@
         <v>0.2</v>
       </c>
       <c r="V30" s="4">
-        <v>-0.08</v>
+        <v>-7.0000000000000007E-2</v>
       </c>
       <c r="W30" s="4">
         <v>-187</v>
@@ -3120,8 +3081,8 @@
         <v>1500</v>
       </c>
       <c r="AA30" s="2">
-        <f t="shared" si="2"/>
-        <v>-16.623333333333335</v>
+        <f t="shared" si="1"/>
+        <v>-16.223333333333336</v>
       </c>
       <c r="AB30" s="1"/>
       <c r="AC30" s="1"/>
@@ -3135,16 +3096,16 @@
       </c>
       <c r="AH30" s="1"/>
       <c r="AI30" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.49944840000000001</v>
       </c>
     </row>
     <row r="31" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>69</v>
+        <v>99</v>
       </c>
       <c r="C31" s="4">
         <v>12</v>
@@ -3174,8 +3135,7 @@
         <v>1200</v>
       </c>
       <c r="N31" s="2">
-        <f t="shared" si="1"/>
-        <v>-15.089999999999998</v>
+        <v>-15.09</v>
       </c>
       <c r="O31" s="1"/>
       <c r="P31" s="4">
@@ -3206,7 +3166,7 @@
         <v>1200</v>
       </c>
       <c r="AA31" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-15.889999999999999</v>
       </c>
       <c r="AB31" s="1"/>
@@ -3221,16 +3181,16 @@
       </c>
       <c r="AH31" s="1"/>
       <c r="AI31" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.5936998</v>
       </c>
     </row>
     <row r="32" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>71</v>
+        <v>101</v>
       </c>
       <c r="C32" s="4">
         <v>5</v>
@@ -3260,8 +3220,7 @@
         <v>1000</v>
       </c>
       <c r="N32" s="2">
-        <f t="shared" si="1"/>
-        <v>-16.566666666666666</v>
+        <v>-16.57</v>
       </c>
       <c r="O32" s="1"/>
       <c r="P32" s="4">
@@ -3289,10 +3248,10 @@
       <c r="X32" s="3"/>
       <c r="Y32" s="3"/>
       <c r="Z32" s="4">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="AA32" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-15.96666666666667</v>
       </c>
       <c r="AB32" s="1"/>
@@ -3307,16 +3266,16 @@
       </c>
       <c r="AH32" s="1"/>
       <c r="AI32" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.7074033999999999</v>
       </c>
     </row>
     <row r="33" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>72</v>
+        <v>102</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>73</v>
+        <v>103</v>
       </c>
       <c r="C33" s="4">
         <v>3</v>
@@ -3346,8 +3305,7 @@
         <v>1500</v>
       </c>
       <c r="N33" s="2">
-        <f t="shared" si="1"/>
-        <v>-19.080000000000002</v>
+        <v>-19.079999999999998</v>
       </c>
       <c r="O33" s="1"/>
       <c r="P33" s="4">
@@ -3378,7 +3336,7 @@
         <v>1500</v>
       </c>
       <c r="AA33" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-14.88</v>
       </c>
       <c r="AB33" s="1"/>
@@ -3393,16 +3351,16 @@
       </c>
       <c r="AH33" s="1"/>
       <c r="AI33" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.70799999999999996</v>
       </c>
     </row>
     <row r="34" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>74</v>
+        <v>104</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="C34" s="4">
         <v>-6</v>
@@ -3432,8 +3390,7 @@
         <v>1500</v>
       </c>
       <c r="N34" s="2">
-        <f t="shared" si="1"/>
-        <v>-20.406666666666666</v>
+        <v>-20.41</v>
       </c>
       <c r="O34" s="1"/>
       <c r="P34" s="4">
@@ -3464,7 +3421,7 @@
         <v>1500</v>
       </c>
       <c r="AA34" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-15.406666666666665</v>
       </c>
       <c r="AB34" s="1"/>
@@ -3479,16 +3436,16 @@
       </c>
       <c r="AH34" s="1"/>
       <c r="AI34" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.86</v>
       </c>
     </row>
     <row r="35" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>76</v>
+        <v>106</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>77</v>
+        <v>107</v>
       </c>
       <c r="C35" s="4">
         <v>0</v>
@@ -3518,8 +3475,7 @@
         <v>2000</v>
       </c>
       <c r="N35" s="2">
-        <f t="shared" si="1"/>
-        <v>-21.206666666666663</v>
+        <v>-21.21</v>
       </c>
       <c r="O35" s="1"/>
       <c r="P35" s="4">
@@ -3550,7 +3506,7 @@
         <v>2000</v>
       </c>
       <c r="AA35" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-15.156666666666665</v>
       </c>
       <c r="AB35" s="1"/>
@@ -3565,16 +3521,16 @@
       </c>
       <c r="AH35" s="1"/>
       <c r="AI35" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.86</v>
       </c>
     </row>
     <row r="36" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>78</v>
+        <v>108</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>79</v>
+        <v>105</v>
       </c>
       <c r="C36" s="4">
         <v>-2</v>
@@ -3604,12 +3560,11 @@
         <v>1500</v>
       </c>
       <c r="N36" s="2">
-        <f t="shared" si="1"/>
-        <v>-20.473333333333333</v>
+        <v>-20.47</v>
       </c>
       <c r="O36" s="1"/>
       <c r="P36" s="4">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="Q36" s="4">
         <v>1.01</v>
@@ -3636,8 +3591,8 @@
         <v>1500</v>
       </c>
       <c r="AA36" s="2">
-        <f t="shared" si="2"/>
-        <v>-16.873333333333331</v>
+        <f t="shared" si="1"/>
+        <v>-17.873333333333331</v>
       </c>
       <c r="AB36" s="1"/>
       <c r="AC36" s="1"/>
@@ -3651,7 +3606,7 @@
       </c>
       <c r="AH36" s="1"/>
       <c r="AI36" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.86</v>
       </c>
     </row>
@@ -3670,7 +3625,6 @@
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
       <c r="N37" s="2">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O37" s="1"/>
@@ -3686,7 +3640,7 @@
       <c r="Y37" s="1"/>
       <c r="Z37" s="1"/>
       <c r="AA37" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AB37" s="1"/>
@@ -3700,10 +3654,10 @@
     </row>
     <row r="38" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>81</v>
+        <v>110</v>
       </c>
       <c r="C38" s="1">
         <v>-1</v>
@@ -3733,15 +3687,14 @@
         <v>0</v>
       </c>
       <c r="N38" s="2">
-        <f t="shared" si="1"/>
-        <v>2.7500000000000004</v>
+        <v>2.75</v>
       </c>
       <c r="O38" s="1"/>
       <c r="P38" s="1">
         <v>1</v>
       </c>
       <c r="Q38" s="1">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="R38" s="1">
         <v>-10</v>
@@ -3765,8 +3718,8 @@
         <v>0</v>
       </c>
       <c r="AA38" s="2">
-        <f t="shared" si="2"/>
-        <v>15.399999999999999</v>
+        <f t="shared" si="1"/>
+        <v>15</v>
       </c>
       <c r="AB38" s="1"/>
       <c r="AC38" s="1"/>
@@ -3776,16 +3729,16 @@
       <c r="AG38" s="1"/>
       <c r="AH38" s="1"/>
       <c r="AI38" s="1">
-        <f t="shared" ref="AI38:AI41" si="4">AF38+AG38*0.038+AH38</f>
+        <f t="shared" ref="AI38:AI41" si="3">AF38+AG38*0.038+AH38</f>
         <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>135</v>
+        <v>111</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>136</v>
+        <v>112</v>
       </c>
       <c r="C39" s="1">
         <v>2</v>
@@ -3811,15 +3764,14 @@
         <v>600</v>
       </c>
       <c r="N39" s="2">
-        <f t="shared" si="1"/>
-        <v>9.8833333333333346</v>
+        <v>9.8800000000000008</v>
       </c>
       <c r="O39" s="1"/>
       <c r="P39" s="1">
         <v>2</v>
       </c>
       <c r="Q39" s="1">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="R39" s="1">
         <v>-9</v>
@@ -3843,8 +3795,8 @@
         <v>600</v>
       </c>
       <c r="AA39" s="2">
-        <f t="shared" si="2"/>
-        <v>15.2</v>
+        <f t="shared" si="1"/>
+        <v>14.799999999999999</v>
       </c>
       <c r="AB39" s="1"/>
       <c r="AC39" s="1"/>
@@ -3857,10 +3809,10 @@
     </row>
     <row r="40" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>82</v>
+        <v>44</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>83</v>
+        <v>45</v>
       </c>
       <c r="C40" s="1">
         <v>-2.5</v>
@@ -3890,15 +3842,14 @@
         <v>500</v>
       </c>
       <c r="N40" s="2">
-        <f t="shared" si="1"/>
-        <v>2.4833333333333334</v>
+        <v>2.48</v>
       </c>
       <c r="O40" s="1"/>
       <c r="P40" s="1">
         <v>1</v>
       </c>
       <c r="Q40" s="1">
-        <v>0.09</v>
+        <v>0.12</v>
       </c>
       <c r="R40" s="1">
         <v>-10</v>
@@ -3922,8 +3873,8 @@
         <v>500</v>
       </c>
       <c r="AA40" s="2">
-        <f t="shared" si="2"/>
-        <v>15.766666666666667</v>
+        <f t="shared" si="1"/>
+        <v>15.166666666666666</v>
       </c>
       <c r="AB40" s="1"/>
       <c r="AC40" s="1"/>
@@ -3933,16 +3884,16 @@
       <c r="AG40" s="1"/>
       <c r="AH40" s="1"/>
       <c r="AI40" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>84</v>
+        <v>46</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>85</v>
+        <v>47</v>
       </c>
       <c r="C41" s="1">
         <v>-2</v>
@@ -3972,15 +3923,14 @@
         <v>500</v>
       </c>
       <c r="N41" s="2">
-        <f t="shared" si="1"/>
-        <v>2.5666666666666664</v>
+        <v>2.57</v>
       </c>
       <c r="O41" s="1"/>
       <c r="P41" s="1">
         <v>0</v>
       </c>
       <c r="Q41" s="1">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="R41" s="1">
         <v>-13</v>
@@ -4004,8 +3954,8 @@
         <v>500</v>
       </c>
       <c r="AA41" s="2">
-        <f t="shared" si="2"/>
-        <v>15.883333333333335</v>
+        <f t="shared" si="1"/>
+        <v>15.483333333333334</v>
       </c>
       <c r="AB41" s="1"/>
       <c r="AC41" s="1"/>
@@ -4015,16 +3965,16 @@
       <c r="AG41" s="1"/>
       <c r="AH41" s="1"/>
       <c r="AI41" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>88</v>
+        <v>113</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>89</v>
+        <v>114</v>
       </c>
       <c r="C42" s="1">
         <v>-0.5</v>
@@ -4054,15 +4004,14 @@
         <v>0</v>
       </c>
       <c r="N42" s="2">
-        <f t="shared" si="1"/>
-        <v>2.2666666666666666</v>
+        <v>2.27</v>
       </c>
       <c r="O42" s="1"/>
       <c r="P42" s="1">
         <v>1</v>
       </c>
       <c r="Q42" s="1">
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="R42" s="1">
         <v>-11</v>
@@ -4086,8 +4035,8 @@
         <v>0</v>
       </c>
       <c r="AA42" s="2">
-        <f t="shared" si="2"/>
-        <v>15.883333333333335</v>
+        <f t="shared" si="1"/>
+        <v>15.283333333333333</v>
       </c>
       <c r="AB42" s="1"/>
       <c r="AC42" s="1"/>
@@ -4100,10 +4049,10 @@
     </row>
     <row r="43" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>91</v>
+        <v>116</v>
       </c>
       <c r="C43" s="1">
         <v>-0.5</v>
@@ -4133,15 +4082,14 @@
         <v>750</v>
       </c>
       <c r="N43" s="2">
-        <f t="shared" si="1"/>
-        <v>2.6666666666666665</v>
+        <v>2.67</v>
       </c>
       <c r="O43" s="1"/>
       <c r="P43" s="1">
         <v>1</v>
       </c>
       <c r="Q43" s="1">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
       <c r="R43" s="1">
         <v>-14</v>
@@ -4165,16 +4113,16 @@
         <v>750</v>
       </c>
       <c r="AA43" s="2">
-        <f t="shared" si="2"/>
-        <v>16.883333333333333</v>
+        <f t="shared" si="1"/>
+        <v>16.283333333333335</v>
       </c>
       <c r="AB43" s="1"/>
       <c r="AC43" s="1">
         <v>4.25</v>
       </c>
       <c r="AD43" s="1">
-        <f t="shared" ref="AD43:AD61" si="5">AC43*0.015</f>
-        <v>6.3750000000000001E-2</v>
+        <f>AC43*0.024</f>
+        <v>0.10200000000000001</v>
       </c>
       <c r="AE43" s="1"/>
       <c r="AF43" s="1"/>
@@ -4184,10 +4132,10 @@
     </row>
     <row r="44" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>92</v>
+        <v>48</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>93</v>
+        <v>49</v>
       </c>
       <c r="C44" s="1">
         <v>-1</v>
@@ -4217,15 +4165,14 @@
         <v>1000</v>
       </c>
       <c r="N44" s="2">
-        <f t="shared" si="1"/>
-        <v>5.6666666666666661</v>
+        <v>5.67</v>
       </c>
       <c r="O44" s="1"/>
       <c r="P44" s="1">
         <v>-1</v>
       </c>
       <c r="Q44" s="1">
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="R44" s="1">
         <v>-15</v>
@@ -4249,16 +4196,16 @@
         <v>1000</v>
       </c>
       <c r="AA44" s="2">
-        <f t="shared" si="2"/>
-        <v>16.850000000000001</v>
+        <f t="shared" si="1"/>
+        <v>16.25</v>
       </c>
       <c r="AB44" s="1"/>
       <c r="AC44" s="1">
         <v>4</v>
       </c>
       <c r="AD44" s="1">
-        <f t="shared" si="5"/>
-        <v>0.06</v>
+        <f t="shared" ref="AD44:AD46" si="4">AC44*0.024</f>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="AE44" s="1"/>
       <c r="AF44" s="1"/>
@@ -4268,10 +4215,10 @@
     </row>
     <row r="45" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="C45" s="1">
         <v>-1</v>
@@ -4301,7 +4248,6 @@
         <v>900</v>
       </c>
       <c r="N45" s="2">
-        <f t="shared" si="1"/>
         <v>4.8499999999999996</v>
       </c>
       <c r="O45" s="1"/>
@@ -4309,7 +4255,7 @@
         <v>-2</v>
       </c>
       <c r="Q45" s="1">
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="R45" s="1">
         <v>-17</v>
@@ -4333,16 +4279,16 @@
         <v>900</v>
       </c>
       <c r="AA45" s="2">
-        <f t="shared" si="2"/>
-        <v>16.850000000000001</v>
+        <f t="shared" si="1"/>
+        <v>16.25</v>
       </c>
       <c r="AB45" s="1"/>
       <c r="AC45" s="1">
         <v>3.9</v>
       </c>
       <c r="AD45" s="1">
-        <f t="shared" si="5"/>
-        <v>5.8499999999999996E-2</v>
+        <f t="shared" si="4"/>
+        <v>9.3600000000000003E-2</v>
       </c>
       <c r="AE45" s="1"/>
       <c r="AF45" s="1"/>
@@ -4352,10 +4298,10 @@
     </row>
     <row r="46" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="C46" s="1">
         <v>-1</v>
@@ -4385,7 +4331,6 @@
         <v>500</v>
       </c>
       <c r="N46" s="2">
-        <f t="shared" si="1"/>
         <v>4.7</v>
       </c>
       <c r="O46" s="1"/>
@@ -4393,7 +4338,7 @@
         <v>-1</v>
       </c>
       <c r="Q46" s="1">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="R46" s="1">
         <v>-13</v>
@@ -4417,16 +4362,16 @@
         <v>500</v>
       </c>
       <c r="AA46" s="2">
-        <f t="shared" si="2"/>
-        <v>16.649999999999999</v>
+        <f t="shared" si="1"/>
+        <v>16.05</v>
       </c>
       <c r="AB46" s="1"/>
       <c r="AC46" s="1">
         <v>3.6</v>
       </c>
       <c r="AD46" s="1">
-        <f t="shared" si="5"/>
-        <v>5.3999999999999999E-2</v>
+        <f t="shared" si="4"/>
+        <v>8.6400000000000005E-2</v>
       </c>
       <c r="AE46" s="1"/>
       <c r="AF46" s="1"/>
@@ -4436,10 +4381,10 @@
     </row>
     <row r="47" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>86</v>
+        <v>50</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>87</v>
+        <v>51</v>
       </c>
       <c r="C47" s="1">
         <v>-4</v>
@@ -4469,18 +4414,17 @@
         <v>1200</v>
       </c>
       <c r="N47" s="2">
-        <f>C47-D47*20-E47*0.8-F47*0.6-H47*15+I47*40+J47/300</f>
-        <v>-6.5000000000000036</v>
+        <v>-6.5</v>
       </c>
       <c r="O47" s="1"/>
       <c r="P47" s="1">
         <v>-3</v>
       </c>
       <c r="Q47" s="1">
-        <v>0.04</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="R47" s="1">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="S47" s="1">
         <v>-22</v>
@@ -4502,7 +4446,7 @@
       </c>
       <c r="AA47" s="2">
         <f>P47-Q47*20-R47*0.8-S47*0.6-U47*15+V47*40+W47/300</f>
-        <v>-3.7000000000000006</v>
+        <v>-2.7000000000000024</v>
       </c>
       <c r="AB47" s="1"/>
       <c r="AC47" s="1"/>
@@ -4518,10 +4462,10 @@
     </row>
     <row r="48" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>98</v>
+        <v>52</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>99</v>
+        <v>53</v>
       </c>
       <c r="C48" s="1">
         <v>-6</v>
@@ -4551,18 +4495,17 @@
         <v>1500</v>
       </c>
       <c r="N48" s="2">
-        <f t="shared" si="1"/>
-        <v>-4.7666666666666684</v>
+        <v>-4.7699999999999996</v>
       </c>
       <c r="O48" s="1"/>
       <c r="P48" s="1">
         <v>-6</v>
       </c>
       <c r="Q48" s="1">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="R48" s="1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="S48" s="1">
         <v>-35</v>
@@ -4583,13 +4526,13 @@
         <v>1500</v>
       </c>
       <c r="AA48" s="2">
-        <f t="shared" si="2"/>
-        <v>1.0833333333333341</v>
+        <f t="shared" si="1"/>
+        <v>2.4833333333333325</v>
       </c>
       <c r="AB48" s="1"/>
       <c r="AC48" s="1"/>
       <c r="AD48" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="AD48:AD61" si="5">AC48*0.015</f>
         <v>0</v>
       </c>
       <c r="AE48" s="1"/>
@@ -4613,7 +4556,6 @@
       <c r="L49" s="1"/>
       <c r="M49" s="1"/>
       <c r="N49" s="2">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O49" s="1"/>
@@ -4629,7 +4571,7 @@
       <c r="Y49" s="1"/>
       <c r="Z49" s="1"/>
       <c r="AA49" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AB49" s="1"/>
@@ -4646,10 +4588,10 @@
     </row>
     <row r="50" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>100</v>
+        <v>121</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>101</v>
+        <v>122</v>
       </c>
       <c r="C50" s="1">
         <v>0</v>
@@ -4679,8 +4621,7 @@
         <v>1000</v>
       </c>
       <c r="N50" s="2">
-        <f t="shared" si="1"/>
-        <v>17.733333333333331</v>
+        <v>17.73</v>
       </c>
       <c r="O50" s="1"/>
       <c r="P50" s="1">
@@ -4711,7 +4652,7 @@
         <v>1000</v>
       </c>
       <c r="AA50" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>16.533333333333331</v>
       </c>
       <c r="AB50" s="1"/>
@@ -4730,10 +4671,10 @@
     </row>
     <row r="51" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>102</v>
+        <v>123</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>103</v>
+        <v>124</v>
       </c>
       <c r="C51" s="1">
         <v>0</v>
@@ -4763,8 +4704,7 @@
         <v>1000</v>
       </c>
       <c r="N51" s="2">
-        <f t="shared" si="1"/>
-        <v>17.466666666666669</v>
+        <v>17.47</v>
       </c>
       <c r="O51" s="1"/>
       <c r="P51" s="1">
@@ -4795,7 +4735,7 @@
         <v>1000</v>
       </c>
       <c r="AA51" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>16.266666666666666</v>
       </c>
       <c r="AB51" s="1"/>
@@ -4827,7 +4767,6 @@
       <c r="L52" s="1"/>
       <c r="M52" s="1"/>
       <c r="N52" s="2">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O52" s="1"/>
@@ -4843,7 +4782,7 @@
       <c r="Y52" s="1"/>
       <c r="Z52" s="1"/>
       <c r="AA52" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AB52" s="1"/>
@@ -4860,10 +4799,10 @@
     </row>
     <row r="53" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>105</v>
+        <v>55</v>
       </c>
       <c r="C53" s="3">
         <v>-6</v>
@@ -4893,8 +4832,7 @@
         <v>2000</v>
       </c>
       <c r="N53" s="2">
-        <f t="shared" si="1"/>
-        <v>8.1666666666666679</v>
+        <v>8.17</v>
       </c>
       <c r="O53" s="1"/>
       <c r="P53" s="3">
@@ -4904,10 +4842,10 @@
         <v>0.26</v>
       </c>
       <c r="R53" s="3">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="S53" s="3">
-        <v>-12</v>
+        <v>-13</v>
       </c>
       <c r="T53" s="3"/>
       <c r="U53" s="3">
@@ -4925,8 +4863,8 @@
         <v>2000</v>
       </c>
       <c r="AA53" s="2">
-        <f t="shared" si="2"/>
-        <v>8.4666666666666668</v>
+        <f t="shared" si="1"/>
+        <v>9.8666666666666671</v>
       </c>
       <c r="AB53" s="1"/>
       <c r="AC53" s="1">
@@ -4944,10 +4882,10 @@
     </row>
     <row r="54" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="C54" s="3">
         <v>-5</v>
@@ -4977,8 +4915,7 @@
         <v>2500</v>
       </c>
       <c r="N54" s="2">
-        <f t="shared" si="1"/>
-        <v>3.1000000000000005</v>
+        <v>3.1</v>
       </c>
       <c r="O54" s="1"/>
       <c r="P54" s="3">
@@ -4988,10 +4925,10 @@
         <v>0.16</v>
       </c>
       <c r="R54" s="3">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="S54" s="3">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="T54" s="3"/>
       <c r="U54" s="3">
@@ -5009,8 +4946,8 @@
         <v>2500</v>
       </c>
       <c r="AA54" s="2">
-        <f t="shared" si="2"/>
-        <v>8.6</v>
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
       <c r="AB54" s="1"/>
       <c r="AC54" s="1">
@@ -5028,10 +4965,10 @@
     </row>
     <row r="55" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>109</v>
+        <v>128</v>
       </c>
       <c r="C55" s="3">
         <v>-4</v>
@@ -5061,8 +4998,7 @@
         <v>1000</v>
       </c>
       <c r="N55" s="2">
-        <f t="shared" si="1"/>
-        <v>5.4999999999999991</v>
+        <v>5.5</v>
       </c>
       <c r="O55" s="1"/>
       <c r="P55" s="3">
@@ -5072,10 +5008,10 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="R55" s="3">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="S55" s="3">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T55" s="3"/>
       <c r="U55" s="3">
@@ -5093,8 +5029,8 @@
         <v>1000</v>
       </c>
       <c r="AA55" s="2">
-        <f t="shared" si="2"/>
-        <v>2.6333333333333329</v>
+        <f t="shared" si="1"/>
+        <v>1.2333333333333327</v>
       </c>
       <c r="AB55" s="1"/>
       <c r="AC55" s="1"/>
@@ -5110,10 +5046,10 @@
     </row>
     <row r="56" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="C56" s="3">
         <v>-8</v>
@@ -5143,8 +5079,7 @@
         <v>1500</v>
       </c>
       <c r="N56" s="2">
-        <f t="shared" si="1"/>
-        <v>-0.76666666666666727</v>
+        <v>-0.77</v>
       </c>
       <c r="O56" s="1"/>
       <c r="P56" s="3">
@@ -5154,10 +5089,10 @@
         <v>0.21</v>
       </c>
       <c r="R56" s="3">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="S56" s="3">
-        <v>-13</v>
+        <v>-14</v>
       </c>
       <c r="T56" s="3"/>
       <c r="U56" s="3">
@@ -5175,8 +5110,8 @@
         <v>1500</v>
       </c>
       <c r="AA56" s="2">
-        <f t="shared" si="2"/>
-        <v>8.8333333333333339</v>
+        <f t="shared" si="1"/>
+        <v>10.233333333333336</v>
       </c>
       <c r="AB56" s="1"/>
       <c r="AC56" s="1">
@@ -5194,10 +5129,10 @@
     </row>
     <row r="57" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>112</v>
+        <v>131</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
       <c r="C57" s="3">
         <v>-8</v>
@@ -5227,8 +5162,7 @@
         <v>1500</v>
       </c>
       <c r="N57" s="2">
-        <f t="shared" si="1"/>
-        <v>-0.76666666666666727</v>
+        <v>-0.77</v>
       </c>
       <c r="O57" s="1"/>
       <c r="P57" s="3">
@@ -5238,10 +5172,10 @@
         <v>0.21</v>
       </c>
       <c r="R57" s="3">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="S57" s="3">
-        <v>-13</v>
+        <v>-14</v>
       </c>
       <c r="T57" s="3"/>
       <c r="U57" s="3">
@@ -5259,8 +5193,8 @@
         <v>1500</v>
       </c>
       <c r="AA57" s="2">
-        <f t="shared" si="2"/>
-        <v>8.8333333333333339</v>
+        <f t="shared" si="1"/>
+        <v>10.233333333333336</v>
       </c>
       <c r="AB57" s="1"/>
       <c r="AC57" s="1"/>
@@ -5276,10 +5210,10 @@
     </row>
     <row r="58" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>114</v>
+        <v>56</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>115</v>
+        <v>57</v>
       </c>
       <c r="C58" s="1">
         <v>-2</v>
@@ -5309,8 +5243,7 @@
         <v>1500</v>
       </c>
       <c r="N58" s="2">
-        <f t="shared" si="1"/>
-        <v>1.6166666666666665</v>
+        <v>1.62</v>
       </c>
       <c r="O58" s="1"/>
       <c r="P58" s="1">
@@ -5320,10 +5253,10 @@
         <v>0.12</v>
       </c>
       <c r="R58" s="1">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="S58" s="1">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="T58" s="1"/>
       <c r="U58" s="1">
@@ -5341,8 +5274,8 @@
         <v>1500</v>
       </c>
       <c r="AA58" s="2">
-        <f t="shared" si="2"/>
-        <v>8.9</v>
+        <f t="shared" si="1"/>
+        <v>10.299999999999999</v>
       </c>
       <c r="AB58" s="1"/>
       <c r="AC58" s="1">
@@ -5360,10 +5293,10 @@
     </row>
     <row r="59" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>116</v>
+        <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>117</v>
+        <v>59</v>
       </c>
       <c r="C59" s="1">
         <v>-4</v>
@@ -5393,8 +5326,7 @@
         <v>2000</v>
       </c>
       <c r="N59" s="2">
-        <f t="shared" si="1"/>
-        <v>4.666666666666667</v>
+        <v>4.67</v>
       </c>
       <c r="O59" s="1"/>
       <c r="P59" s="1">
@@ -5404,10 +5336,10 @@
         <v>0.15</v>
       </c>
       <c r="R59" s="1">
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="S59" s="1">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="T59" s="1"/>
       <c r="U59" s="1">
@@ -5425,8 +5357,8 @@
         <v>2000</v>
       </c>
       <c r="AA59" s="2">
-        <f t="shared" si="2"/>
-        <v>8.9833333333333325</v>
+        <f t="shared" si="1"/>
+        <v>10.383333333333333</v>
       </c>
       <c r="AB59" s="1"/>
       <c r="AC59" s="1"/>
@@ -5442,10 +5374,10 @@
     </row>
     <row r="60" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>118</v>
+        <v>60</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>119</v>
+        <v>61</v>
       </c>
       <c r="C60" s="1">
         <v>-6</v>
@@ -5475,8 +5407,7 @@
         <v>3000</v>
       </c>
       <c r="N60" s="2">
-        <f t="shared" si="1"/>
-        <v>6.9166666666666661</v>
+        <v>6.92</v>
       </c>
       <c r="O60" s="1"/>
       <c r="P60" s="1">
@@ -5486,10 +5417,10 @@
         <v>0.18</v>
       </c>
       <c r="R60" s="1">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="S60" s="1">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="T60" s="1"/>
       <c r="U60" s="1">
@@ -5507,8 +5438,8 @@
         <v>3000</v>
       </c>
       <c r="AA60" s="2">
-        <f t="shared" si="2"/>
-        <v>8.9166666666666661</v>
+        <f t="shared" si="1"/>
+        <v>10.316666666666668</v>
       </c>
       <c r="AB60" s="1"/>
       <c r="AC60" s="1">
@@ -5526,10 +5457,10 @@
     </row>
     <row r="61" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>120</v>
+        <v>62</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>121</v>
+        <v>63</v>
       </c>
       <c r="C61" s="3">
         <v>-3</v>
@@ -5559,8 +5490,7 @@
         <v>700</v>
       </c>
       <c r="N61" s="2">
-        <f t="shared" si="1"/>
-        <v>-7.7499999999999991</v>
+        <v>-7.75</v>
       </c>
       <c r="O61" s="1"/>
       <c r="P61" s="3">
@@ -5570,10 +5500,10 @@
         <v>0.05</v>
       </c>
       <c r="R61" s="3">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="S61" s="3">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="T61" s="3"/>
       <c r="U61" s="3">
@@ -5591,8 +5521,8 @@
         <v>700</v>
       </c>
       <c r="AA61" s="2">
-        <f t="shared" si="2"/>
-        <v>2.35</v>
+        <f t="shared" si="1"/>
+        <v>3.75</v>
       </c>
       <c r="AB61" s="1"/>
       <c r="AC61" s="1">
@@ -5610,10 +5540,10 @@
     </row>
     <row r="62" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>122</v>
+        <v>64</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>123</v>
+        <v>65</v>
       </c>
       <c r="C62" s="3">
         <v>-3</v>
@@ -5643,8 +5573,7 @@
         <v>300</v>
       </c>
       <c r="N62" s="2">
-        <f t="shared" si="1"/>
-        <v>-4.9499999999999975</v>
+        <v>-4.95</v>
       </c>
       <c r="O62" s="1"/>
       <c r="P62" s="3">
@@ -5654,10 +5583,10 @@
         <v>0.04</v>
       </c>
       <c r="R62" s="3">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="S62" s="3">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="T62" s="3"/>
       <c r="U62" s="3">
@@ -5675,8 +5604,8 @@
         <v>300</v>
       </c>
       <c r="AA62" s="2">
-        <f t="shared" si="2"/>
-        <v>9.3000000000000007</v>
+        <f t="shared" si="1"/>
+        <v>10.700000000000001</v>
       </c>
       <c r="AB62" s="1"/>
       <c r="AC62" s="1"/>
@@ -5689,10 +5618,10 @@
     </row>
     <row r="63" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="C63" s="3">
         <v>-6</v>
@@ -5722,8 +5651,7 @@
         <v>1000</v>
       </c>
       <c r="N63" s="2">
-        <f t="shared" si="1"/>
-        <v>8.5666666666666664</v>
+        <v>8.57</v>
       </c>
       <c r="O63" s="1"/>
       <c r="P63" s="3">
@@ -5733,10 +5661,10 @@
         <v>0.18</v>
       </c>
       <c r="R63" s="3">
-        <v>-12</v>
+        <v>-13</v>
       </c>
       <c r="S63" s="3">
-        <v>-12</v>
+        <v>-13</v>
       </c>
       <c r="T63" s="3"/>
       <c r="U63" s="3">
@@ -5754,8 +5682,8 @@
         <v>1000</v>
       </c>
       <c r="AA63" s="2">
-        <f t="shared" si="2"/>
-        <v>11.55</v>
+        <f t="shared" si="1"/>
+        <v>12.950000000000001</v>
       </c>
       <c r="AB63" s="1"/>
       <c r="AC63" s="1">
@@ -5773,10 +5701,10 @@
     </row>
     <row r="64" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="C64" s="3">
         <v>-0.5</v>
@@ -5796,7 +5724,6 @@
         <v>200</v>
       </c>
       <c r="N64" s="2">
-        <f t="shared" si="1"/>
         <v>-1.1000000000000001</v>
       </c>
       <c r="O64" s="1"/>
@@ -5818,7 +5745,7 @@
         <v>200</v>
       </c>
       <c r="AA64" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-0.6</v>
       </c>
       <c r="AB64" s="1"/>
@@ -5845,7 +5772,6 @@
       <c r="L65" s="3"/>
       <c r="M65" s="3"/>
       <c r="N65" s="2">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O65" s="1"/>
@@ -5861,7 +5787,7 @@
       <c r="Y65" s="3"/>
       <c r="Z65" s="3"/>
       <c r="AA65" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AB65" s="1"/>
@@ -5875,10 +5801,10 @@
     </row>
     <row r="66" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>128</v>
+        <v>66</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>129</v>
+        <v>67</v>
       </c>
       <c r="C66" s="1">
         <v>-1</v>
@@ -5906,8 +5832,7 @@
         <v>500</v>
       </c>
       <c r="N66" s="2">
-        <f t="shared" si="1"/>
-        <v>-2.9666666666666668</v>
+        <v>-2.97</v>
       </c>
       <c r="O66" s="1"/>
       <c r="P66" s="1">
@@ -5938,7 +5863,7 @@
         <v>500</v>
       </c>
       <c r="AA66" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-2.2833333333333332</v>
       </c>
       <c r="AB66" s="1"/>
@@ -5952,10 +5877,10 @@
     </row>
     <row r="67" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>130</v>
+        <v>68</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>131</v>
+        <v>69</v>
       </c>
       <c r="C67" s="1">
         <v>-1.5</v>
@@ -5985,8 +5910,7 @@
         <v>750</v>
       </c>
       <c r="N67" s="2">
-        <f t="shared" si="1"/>
-        <v>-1.4999999999999998</v>
+        <v>-1.5</v>
       </c>
       <c r="O67" s="1"/>
       <c r="P67" s="1">
@@ -6017,7 +5941,7 @@
         <v>750</v>
       </c>
       <c r="AA67" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>-4.3666666666666663</v>
       </c>
       <c r="AB67" s="1"/>
@@ -6031,10 +5955,10 @@
     </row>
     <row r="68" spans="1:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>132</v>
+        <v>70</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>133</v>
+        <v>71</v>
       </c>
       <c r="C68" s="1">
         <v>-3</v>
@@ -6064,8 +5988,7 @@
         <v>1000</v>
       </c>
       <c r="N68" s="2">
-        <f t="shared" si="1"/>
-        <v>-2.5333333333333332</v>
+        <v>-2.5299999999999998</v>
       </c>
       <c r="O68" s="1"/>
       <c r="P68" s="1">
@@ -6085,7 +6008,7 @@
         <v>0.2</v>
       </c>
       <c r="V68" s="1">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="W68" s="1">
         <v>80</v>
@@ -6096,8 +6019,8 @@
         <v>1000</v>
       </c>
       <c r="AA68" s="2">
-        <f t="shared" si="2"/>
-        <v>-7.5333333333333341</v>
+        <f t="shared" si="1"/>
+        <v>-7.9333333333333345</v>
       </c>
       <c r="AB68" s="1"/>
       <c r="AC68" s="1"/>
@@ -6241,9 +6164,7 @@
       <c r="S72" s="1"/>
       <c r="T72" s="1"/>
       <c r="U72" s="1"/>
-      <c r="V72" s="1" t="s">
-        <v>134</v>
-      </c>
+      <c r="V72" s="1"/>
       <c r="W72" s="1"/>
       <c r="X72" s="1"/>
       <c r="Y72" s="1"/>
@@ -41599,7 +41520,6 @@
       <formula>P3&lt;&gt;C3</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="portrait"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
nerf fal 8" barrel and other short barrels
</commit_message>
<xml_diff>
--- a/changes/308-barrels-muzzles.xlsx
+++ b/changes/308-barrels-muzzles.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84D2787F-9C7A-4597-94BF-1B9475D36796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E47B1B07-FB8E-47EA-8D7B-3BBEB492CA9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1289,7 +1289,7 @@
         <v>0.45</v>
       </c>
       <c r="I13">
-        <v>-0.08</v>
+        <v>-0.09</v>
       </c>
       <c r="J13">
         <v>-331</v>
@@ -1299,7 +1299,7 @@
       </c>
       <c r="N13" s="2">
         <f t="shared" si="0"/>
-        <v>-28.853333333333328</v>
+        <v>-29.25333333333333</v>
       </c>
       <c r="O13" s="1"/>
       <c r="P13" s="1"/>
@@ -1635,7 +1635,7 @@
         <v>98</v>
       </c>
       <c r="C21">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D21">
         <v>0.49</v>
@@ -1647,10 +1647,10 @@
         <v>9</v>
       </c>
       <c r="H21">
-        <v>0.25</v>
+        <v>0.35</v>
       </c>
       <c r="I21">
-        <v>-0.08</v>
+        <v>-0.09</v>
       </c>
       <c r="J21">
         <v>-158</v>
@@ -1660,7 +1660,7 @@
       </c>
       <c r="N21" s="2">
         <f t="shared" si="0"/>
-        <v>-13.876666666666669</v>
+        <v>-18.776666666666667</v>
       </c>
       <c r="O21" s="1"/>
       <c r="P21" s="1"/>
@@ -1686,7 +1686,7 @@
         <v>99</v>
       </c>
       <c r="C22">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D22">
         <v>0.67</v>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="N22" s="2">
         <f t="shared" si="0"/>
-        <v>-19.886666666666667</v>
+        <v>-18.886666666666667</v>
       </c>
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
@@ -2071,7 +2071,7 @@
         <v>7</v>
       </c>
       <c r="H30">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="I30">
         <v>-7.0000000000000007E-2</v>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="N30" s="2">
         <f t="shared" si="0"/>
-        <v>-16.223333333333336</v>
+        <v>-16.973333333333336</v>
       </c>
       <c r="O30" s="1"/>
       <c r="P30" s="1"/>

</xml_diff>

<commit_message>
i forgor the sd
</commit_message>
<xml_diff>
--- a/changes/308-barrels-muzzles.xlsx
+++ b/changes/308-barrels-muzzles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-dev\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07855C36-F8FF-4EEF-AACC-A71A8C347BDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8138B90-9EF3-473C-BD3B-E69B6A21091B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1460,9 +1460,12 @@
       <c r="J16">
         <v>90</v>
       </c>
+      <c r="M16">
+        <v>-0.19</v>
+      </c>
       <c r="O16" s="2">
         <f t="shared" si="0"/>
-        <v>7.9000000000000012</v>
+        <v>8.8500000000000014</v>
       </c>
       <c r="P16" s="1"/>
       <c r="Q16" s="1"/>
@@ -1550,6 +1553,9 @@
       </c>
       <c r="J18">
         <v>50</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
       </c>
       <c r="N18">
         <v>0</v>

</xml_diff>